<commit_message>
Daily slate 2026-03-31 [auto]
</commit_message>
<xml_diff>
--- a/CBB/step6_ranked_wcbb.xlsx
+++ b/CBB/step6_ranked_wcbb.xlsx
@@ -963,7 +963,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD2" t="n">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD3" t="n">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD4" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD5" t="n">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD6" t="n">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD7" t="n">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD8" t="n">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD9" t="n">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD10" t="n">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD11" t="n">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD12" t="n">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD13" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD14" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD15" t="n">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD16" t="n">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD17" t="n">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD18" t="n">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD19" t="n">
@@ -6199,7 +6199,7 @@
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD20" t="n">
@@ -6491,7 +6491,7 @@
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD21" t="n">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD22" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD23" t="n">
@@ -7379,7 +7379,7 @@
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD24" t="n">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD25" t="n">
@@ -7971,7 +7971,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD26" t="n">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD27" t="n">
@@ -8551,7 +8551,7 @@
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD28" t="n">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD29" t="n">
@@ -9131,7 +9131,7 @@
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD30" t="n">
@@ -9421,7 +9421,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD31" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD32" t="n">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD33" t="n">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="AC34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD34" t="n">
@@ -10537,7 +10537,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD35" t="n">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="AC36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD36" t="n">
@@ -11945,7 +11945,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD2" t="n">
@@ -12241,7 +12241,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD3" t="n">
@@ -12537,7 +12537,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD4" t="n">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD5" t="n">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD6" t="n">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD7" t="n">
@@ -13721,7 +13721,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD8" t="n">
@@ -14017,7 +14017,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD9" t="n">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD10" t="n">
@@ -14565,7 +14565,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD11" t="n">
@@ -14857,7 +14857,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD12" t="n">
@@ -15153,7 +15153,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD13" t="n">
@@ -15449,7 +15449,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD14" t="n">
@@ -15745,7 +15745,7 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD15" t="n">
@@ -16041,7 +16041,7 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD16" t="n">
@@ -16337,7 +16337,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD17" t="n">
@@ -16633,7 +16633,7 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD18" t="n">
@@ -16909,7 +16909,7 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD19" t="n">
@@ -17181,7 +17181,7 @@
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD20" t="n">
@@ -17473,7 +17473,7 @@
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD21" t="n">
@@ -17769,7 +17769,7 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD22" t="n">
@@ -18065,7 +18065,7 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD23" t="n">
@@ -18361,7 +18361,7 @@
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD24" t="n">
@@ -18657,7 +18657,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD25" t="n">
@@ -18953,7 +18953,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD26" t="n">
@@ -19243,7 +19243,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD27" t="n">
@@ -19533,7 +19533,7 @@
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD28" t="n">
@@ -19823,7 +19823,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD29" t="n">
@@ -20113,7 +20113,7 @@
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD30" t="n">
@@ -20403,7 +20403,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD31" t="n">
@@ -20693,7 +20693,7 @@
       </c>
       <c r="AC32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD32" t="n">
@@ -20963,7 +20963,7 @@
       </c>
       <c r="AC33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD33" t="n">
@@ -21249,7 +21249,7 @@
       </c>
       <c r="AC34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD34" t="n">
@@ -21519,7 +21519,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD35" t="n">
@@ -21805,7 +21805,7 @@
       </c>
       <c r="AC36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="AD36" t="n">

</xml_diff>

<commit_message>
Daily slate 2026-04-02 [auto]
</commit_message>
<xml_diff>
--- a/CBB/step6_ranked_wcbb.xlsx
+++ b/CBB/step6_ranked_wcbb.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ELIGIBLE" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIER_A" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIER_B" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIER_D" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIER_C" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TIER_D" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2607,27 +2608,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11036007</t>
+          <t>11037367</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>224015</t>
+          <t>232538</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>sarah strong|CONN</t>
+          <t>azzi fudd|CONN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sarah Strong</t>
+          <t>Azzi Fudd</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>sarah strong</t>
+          <t>azzi fudd</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2652,27 +2653,27 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Pts+Rebs</t>
+          <t>3-PT Made</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>pr</t>
+          <t>fg3m</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Goblin</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -2697,12 +2698,12 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Pts+Rebs</t>
+          <t>3-PT Made</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>goblin</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -2712,7 +2713,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -2732,27 +2733,27 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>23.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr"/>
@@ -2762,37 +2763,37 @@
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="AU6" t="inlineStr">
@@ -2802,28 +2803,28 @@
       </c>
       <c r="AV6" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="AX6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AY6" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="AZ6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="BB6" t="inlineStr">
@@ -2833,19 +2834,19 @@
       </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="BD6" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="BE6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="BG6" t="inlineStr">
         <is>
@@ -2865,16 +2866,16 @@
         </is>
       </c>
       <c r="BL6" t="n">
-        <v>27</v>
+        <v>2.8</v>
       </c>
       <c r="BM6" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="BN6" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="BO6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BP6" t="inlineStr">
         <is>
@@ -2882,47 +2883,51 @@
         </is>
       </c>
       <c r="BQ6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR6" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="BR6" t="inlineStr">
+        <is>
+          <t>VOID_LOW_MINUTES_NON_A</t>
+        </is>
+      </c>
       <c r="BS6" t="n">
         <v>0</v>
       </c>
       <c r="BT6" t="n">
-        <v>27</v>
+        <v>2.8</v>
       </c>
       <c r="BU6" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="BV6" t="n">
-        <v>2.17895874348904</v>
+        <v>1.249832603063641</v>
       </c>
       <c r="BW6" t="n">
         <v>0</v>
       </c>
       <c r="BX6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BY6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BZ6" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="CA6" t="n">
         <v>0</v>
       </c>
       <c r="CB6" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.5226307237858404</v>
       </c>
       <c r="CC6" t="n">
-        <v>0.5880681872367859</v>
+        <v>0.6728972196578979</v>
       </c>
       <c r="CD6" t="n">
-        <v>0.08806818723678589</v>
+        <v>0.1728972196578979</v>
       </c>
       <c r="CE6" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.5226307237858404</v>
       </c>
       <c r="CF6" t="inlineStr">
         <is>
@@ -2951,7 +2956,7 @@
         </is>
       </c>
       <c r="CL6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="CM6" t="inlineStr">
         <is>
@@ -2967,36 +2972,36 @@
         <v>2</v>
       </c>
       <c r="CP6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CQ6" t="n">
         <v>1</v>
       </c>
       <c r="CR6" t="n">
-        <v>24.5</v>
+        <v>1.5</v>
       </c>
       <c r="CS6" t="inlineStr"/>
       <c r="CT6" t="inlineStr"/>
       <c r="CU6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="CV6" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="CW6" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="CX6" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="CY6" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.5226307237858404</v>
       </c>
       <c r="CZ6" t="n">
         <v>1</v>
       </c>
       <c r="DA6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="DB6" t="inlineStr"/>
       <c r="DC6" t="n">
@@ -3006,7 +3011,7 @@
         <v>2</v>
       </c>
       <c r="DE6" t="n">
-        <v>1.216216216216216</v>
+        <v>1.272727272727273</v>
       </c>
       <c r="DF6" t="n">
         <v>1</v>
@@ -3015,27 +3020,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11037367</t>
+          <t>11036007</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>232538</t>
+          <t>224015</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>azzi fudd|CONN</t>
+          <t>sarah strong|CONN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Azzi Fudd</t>
+          <t>Sarah Strong</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>azzi fudd</t>
+          <t>sarah strong</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -3060,27 +3065,27 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>3-PT Made</t>
+          <t>Pts+Rebs</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>fg3m</t>
+          <t>pr</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Goblin</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -3105,12 +3110,12 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>3-PT Made</t>
+          <t>Pts+Rebs</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>goblin</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -3120,7 +3125,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -3140,27 +3145,27 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>28.0</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>23.0</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr"/>
@@ -3170,37 +3175,37 @@
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>2.8</t>
+          <t>27.0</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>30.2</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>30.2</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
@@ -3210,28 +3215,28 @@
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="AX7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="AY7" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="AZ7" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="BA7" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="BB7" t="inlineStr">
@@ -3241,19 +3246,19 @@
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="BD7" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="BE7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="BG7" t="inlineStr">
         <is>
@@ -3273,16 +3278,16 @@
         </is>
       </c>
       <c r="BL7" t="n">
-        <v>2.8</v>
+        <v>27</v>
       </c>
       <c r="BM7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="BN7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="BO7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BP7" t="inlineStr">
         <is>
@@ -3290,51 +3295,47 @@
         </is>
       </c>
       <c r="BQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR7" t="inlineStr">
-        <is>
-          <t>VOID_LOW_MINUTES_NON_A</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="n">
         <v>0</v>
       </c>
       <c r="BT7" t="n">
-        <v>2.8</v>
+        <v>27</v>
       </c>
       <c r="BU7" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="BV7" t="n">
-        <v>1.249832603063641</v>
+        <v>1.411489234785374</v>
       </c>
       <c r="BW7" t="n">
         <v>0</v>
       </c>
       <c r="BX7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="BY7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="BZ7" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="CA7" t="n">
         <v>0</v>
       </c>
       <c r="CB7" t="n">
-        <v>0.5226307237858404</v>
+        <v>0.4484641144988664</v>
       </c>
       <c r="CC7" t="n">
-        <v>0.6728972196578979</v>
+        <v>0.5880681872367859</v>
       </c>
       <c r="CD7" t="n">
-        <v>0.1728972196578979</v>
+        <v>0.08806818723678589</v>
       </c>
       <c r="CE7" t="n">
-        <v>0.5226307237858404</v>
+        <v>0.4484641144988664</v>
       </c>
       <c r="CF7" t="inlineStr">
         <is>
@@ -3354,7 +3355,7 @@
       </c>
       <c r="CJ7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="CK7" t="inlineStr">
@@ -3363,7 +3364,7 @@
         </is>
       </c>
       <c r="CL7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="CM7" t="inlineStr">
         <is>
@@ -3376,39 +3377,39 @@
         </is>
       </c>
       <c r="CO7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CP7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CQ7" t="n">
         <v>1</v>
       </c>
       <c r="CR7" t="n">
-        <v>1.5</v>
+        <v>25.5</v>
       </c>
       <c r="CS7" t="inlineStr"/>
       <c r="CT7" t="inlineStr"/>
       <c r="CU7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="CV7" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="CW7" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="CX7" t="n">
-        <v>0.8666666666666666</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="CY7" t="n">
-        <v>0.5226307237858404</v>
+        <v>0.4484641144988664</v>
       </c>
       <c r="CZ7" t="n">
         <v>1</v>
       </c>
       <c r="DA7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="DB7" t="inlineStr"/>
       <c r="DC7" t="n">
@@ -3418,7 +3419,7 @@
         <v>2</v>
       </c>
       <c r="DE7" t="n">
-        <v>1.272727272727273</v>
+        <v>1.216216216216216</v>
       </c>
       <c r="DF7" t="n">
         <v>1</v>
@@ -46814,7 +46815,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -46854,7 +46855,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
@@ -47010,10 +47011,10 @@
         <v>27</v>
       </c>
       <c r="BM6" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="BN6" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="BO6" t="n">
         <v>0</v>
@@ -47034,10 +47035,10 @@
         <v>27</v>
       </c>
       <c r="BU6" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="BV6" t="n">
-        <v>2.17895874348904</v>
+        <v>1.411489234785374</v>
       </c>
       <c r="BW6" t="n">
         <v>0</v>
@@ -47049,13 +47050,13 @@
         <v>0.8</v>
       </c>
       <c r="BZ6" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="CA6" t="n">
         <v>0</v>
       </c>
       <c r="CB6" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.4484641144988664</v>
       </c>
       <c r="CC6" t="n">
         <v>0.5880681872367859</v>
@@ -47064,7 +47065,7 @@
         <v>0.08806818723678589</v>
       </c>
       <c r="CE6" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.4484641144988664</v>
       </c>
       <c r="CF6" t="inlineStr">
         <is>
@@ -47084,7 +47085,7 @@
       </c>
       <c r="CJ6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="CK6" t="inlineStr">
@@ -47106,7 +47107,7 @@
         </is>
       </c>
       <c r="CO6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CP6" t="n">
         <v>1</v>
@@ -47115,7 +47116,7 @@
         <v>1</v>
       </c>
       <c r="CR6" t="n">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="CS6" t="inlineStr"/>
       <c r="CT6" t="inlineStr"/>
@@ -47126,13 +47127,13 @@
         <v>0.8</v>
       </c>
       <c r="CW6" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="CX6" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.05882352941176471</v>
       </c>
       <c r="CY6" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.4484641144988664</v>
       </c>
       <c r="CZ6" t="n">
         <v>1</v>
@@ -49363,7 +49364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF3"/>
+  <dimension ref="A1:DF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -49921,27 +49922,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11036007</t>
+          <t>11037367</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>224015</t>
+          <t>232538</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>sarah strong|CONN</t>
+          <t>azzi fudd|CONN</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sarah Strong</t>
+          <t>Azzi Fudd</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>sarah strong</t>
+          <t>azzi fudd</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -49966,27 +49967,27 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Pts+Rebs</t>
+          <t>3-PT Made</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>pr</t>
+          <t>fg3m</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Goblin</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -50011,12 +50012,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Pts+Rebs</t>
+          <t>3-PT Made</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>standard</t>
+          <t>goblin</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -50026,7 +50027,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -50046,27 +50047,27 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>28.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>23.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>26.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr"/>
@@ -50076,37 +50077,37 @@
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>27.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>30.2</t>
+          <t>29.4</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="AU2" t="inlineStr">
@@ -50116,28 +50117,28 @@
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="AX2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AY2" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="AZ2" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="BB2" t="inlineStr">
@@ -50147,19 +50148,19 @@
       </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="BE2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BF2" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="BG2" t="inlineStr">
         <is>
@@ -50179,16 +50180,16 @@
         </is>
       </c>
       <c r="BL2" t="n">
-        <v>27</v>
+        <v>2.8</v>
       </c>
       <c r="BM2" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="BN2" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="BO2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BP2" t="inlineStr">
         <is>
@@ -50196,47 +50197,51 @@
         </is>
       </c>
       <c r="BQ2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR2" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>VOID_LOW_MINUTES_NON_A</t>
+        </is>
+      </c>
       <c r="BS2" t="n">
         <v>0</v>
       </c>
       <c r="BT2" t="n">
-        <v>27</v>
+        <v>2.8</v>
       </c>
       <c r="BU2" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="BV2" t="n">
-        <v>2.17895874348904</v>
+        <v>1.249832603063641</v>
       </c>
       <c r="BW2" t="n">
         <v>0</v>
       </c>
       <c r="BX2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BY2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="BZ2" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="CA2" t="n">
         <v>0</v>
       </c>
       <c r="CB2" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.5226307237858404</v>
       </c>
       <c r="CC2" t="n">
-        <v>0.5880681872367859</v>
+        <v>0.6728972196578979</v>
       </c>
       <c r="CD2" t="n">
-        <v>0.08806818723678589</v>
+        <v>0.1728972196578979</v>
       </c>
       <c r="CE2" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.5226307237858404</v>
       </c>
       <c r="CF2" t="inlineStr">
         <is>
@@ -50265,7 +50270,7 @@
         </is>
       </c>
       <c r="CL2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="CM2" t="inlineStr">
         <is>
@@ -50281,36 +50286,36 @@
         <v>2</v>
       </c>
       <c r="CP2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CQ2" t="n">
         <v>1</v>
       </c>
       <c r="CR2" t="n">
-        <v>24.5</v>
+        <v>1.5</v>
       </c>
       <c r="CS2" t="inlineStr"/>
       <c r="CT2" t="inlineStr"/>
       <c r="CU2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="CV2" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="CW2" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="CX2" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.8666666666666666</v>
       </c>
       <c r="CY2" t="n">
-        <v>0.6290977003349064</v>
+        <v>0.5226307237858404</v>
       </c>
       <c r="CZ2" t="n">
         <v>1</v>
       </c>
       <c r="DA2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="DB2" t="inlineStr"/>
       <c r="DC2" t="n">
@@ -50320,421 +50325,9 @@
         <v>2</v>
       </c>
       <c r="DE2" t="n">
-        <v>1.216216216216216</v>
+        <v>1.272727272727273</v>
       </c>
       <c r="DF2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>11037367</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>232538</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>azzi fudd|CONN</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Azzi Fudd</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>azzi fudd</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CONN</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>SCAR</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>CONN</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>SCAR</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>3-PT Made</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>fg3m</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Goblin</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>2026-04-03T19:00:00.000-04:00</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>148432</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>176</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>CONN</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>3-PT Made</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>goblin</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Full</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>8.0</t>
-        </is>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>29.4</t>
-        </is>
-      </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="AT3" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="AU3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AV3" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="AX3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AY3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="BE3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="BH3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="BL3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="BM3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="BN3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="BO3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BP3" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="BQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR3" t="inlineStr">
-        <is>
-          <t>VOID_LOW_MINUTES_NON_A</t>
-        </is>
-      </c>
-      <c r="BS3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BT3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="BU3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="BV3" t="n">
-        <v>1.249832603063641</v>
-      </c>
-      <c r="BW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BX3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="BY3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="BZ3" t="n">
-        <v>0.8666666666666666</v>
-      </c>
-      <c r="CA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB3" t="n">
-        <v>0.5226307237858404</v>
-      </c>
-      <c r="CC3" t="n">
-        <v>0.6728972196578979</v>
-      </c>
-      <c r="CD3" t="n">
-        <v>0.1728972196578979</v>
-      </c>
-      <c r="CE3" t="n">
-        <v>0.5226307237858404</v>
-      </c>
-      <c r="CF3" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="CG3" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="CH3" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="CI3" t="inlineStr">
-        <is>
-          <t>No spread data: 0.97x default</t>
-        </is>
-      </c>
-      <c r="CJ3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="CK3" t="inlineStr">
-        <is>
-          <t>SCAR</t>
-        </is>
-      </c>
-      <c r="CL3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="CM3" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="CN3" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="CO3" t="n">
-        <v>2</v>
-      </c>
-      <c r="CP3" t="n">
-        <v>2</v>
-      </c>
-      <c r="CQ3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CR3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="CS3" t="inlineStr"/>
-      <c r="CT3" t="inlineStr"/>
-      <c r="CU3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="CV3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="CW3" t="n">
-        <v>0.8666666666666666</v>
-      </c>
-      <c r="CX3" t="n">
-        <v>0.8666666666666666</v>
-      </c>
-      <c r="CY3" t="n">
-        <v>0.5226307237858404</v>
-      </c>
-      <c r="CZ3" t="n">
-        <v>1</v>
-      </c>
-      <c r="DA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="n">
-        <v>1</v>
-      </c>
-      <c r="DD3" t="n">
-        <v>2</v>
-      </c>
-      <c r="DE3" t="n">
-        <v>1.272727272727273</v>
-      </c>
-      <c r="DF3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -50744,6 +50337,980 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:DF2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>proj_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>player_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cbb_player_key</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>player_norm</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>team_abbr</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>opp_team_abbr</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pp_team</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>pp_opp_team</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>prop_type</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>prop_norm</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>pick_type</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>pp_game_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>league_id</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>team</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>stat_type</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>odds_type</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>line_num</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>opp_def_rank</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>opp_def_ppg</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>opp_def_tier</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>def_tier</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>OVERALL_DEF_RANK</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>stat_status</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>games_used</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>stat_g1</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>stat_g2</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>stat_g3</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>stat_g4</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>stat_g5</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>stat_g6</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>stat_g7</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>stat_g8</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>stat_g9</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>stat_g10</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>stat_last5_avg</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>stat_last10_avg</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>stat_season_avg</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>min_last5_avg</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>min_season_avg</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>line_hits_over_5</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>line_hits_under_5</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>line_hits_push_5</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_over_5</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_under_5</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_over_ou_5</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_under_ou_5</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>line_hits_over_10</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>line_hits_under_10</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>line_hits_push_10</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_over_10</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_under_10</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_over_ou_10</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>line_hit_rate_under_ou_10</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>model_dir_5</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>usage_boost</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>usage_boost_proj</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>usage_boost_reason</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>usage_boost_source</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>projection</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>abs_edge</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>forced_over_only</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>bet_direction</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>eligible</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>void_reason</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>def_adj</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>projection_adj</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>edge_adj</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>edge_adj_dr</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>def_rank_signal</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>line_hit_rate</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>composite_hit_rate</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>avg_vs_line</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>usage_bonus</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>rank_score</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>ml_prob</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>ml_edge</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>final_score</t>
+        </is>
+      </c>
+      <c r="CF1" t="inlineStr">
+        <is>
+          <t>consistency_grade</t>
+        </is>
+      </c>
+      <c r="CG1" t="inlineStr">
+        <is>
+          <t>consistency_multiplier</t>
+        </is>
+      </c>
+      <c r="CH1" t="inlineStr">
+        <is>
+          <t>game_script_mult</t>
+        </is>
+      </c>
+      <c r="CI1" t="inlineStr">
+        <is>
+          <t>game_script_note</t>
+        </is>
+      </c>
+      <c r="CJ1" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="CK1" t="inlineStr">
+        <is>
+          <t>opp</t>
+        </is>
+      </c>
+      <c r="CL1" t="inlineStr">
+        <is>
+          <t>hit_rate</t>
+        </is>
+      </c>
+      <c r="CM1" t="inlineStr">
+        <is>
+          <t>final_bet_direction</t>
+        </is>
+      </c>
+      <c r="CN1" t="inlineStr">
+        <is>
+          <t>recommended_side</t>
+        </is>
+      </c>
+      <c r="CO1" t="inlineStr">
+        <is>
+          <t>tier_encoded</t>
+        </is>
+      </c>
+      <c r="CP1" t="inlineStr">
+        <is>
+          <t>pick_type_encoded</t>
+        </is>
+      </c>
+      <c r="CQ1" t="inlineStr">
+        <is>
+          <t>direction_encoded</t>
+        </is>
+      </c>
+      <c r="CR1" t="inlineStr">
+        <is>
+          <t>line_score</t>
+        </is>
+      </c>
+      <c r="CS1" t="inlineStr">
+        <is>
+          <t>def_rank</t>
+        </is>
+      </c>
+      <c r="CT1" t="inlineStr">
+        <is>
+          <t>def_tier_encoded</t>
+        </is>
+      </c>
+      <c r="CU1" t="inlineStr">
+        <is>
+          <t>hit_rate_L5</t>
+        </is>
+      </c>
+      <c r="CV1" t="inlineStr">
+        <is>
+          <t>hit_rate_L10</t>
+        </is>
+      </c>
+      <c r="CW1" t="inlineStr">
+        <is>
+          <t>avg_L5_vs_line</t>
+        </is>
+      </c>
+      <c r="CX1" t="inlineStr">
+        <is>
+          <t>avg_L10_vs_line</t>
+        </is>
+      </c>
+      <c r="CY1" t="inlineStr">
+        <is>
+          <t>prop_score</t>
+        </is>
+      </c>
+      <c r="CZ1" t="inlineStr">
+        <is>
+          <t>sport_encoded</t>
+        </is>
+      </c>
+      <c r="DA1" t="inlineStr">
+        <is>
+          <t>minutes_tier</t>
+        </is>
+      </c>
+      <c r="DB1" t="inlineStr">
+        <is>
+          <t>minutes_cv</t>
+        </is>
+      </c>
+      <c r="DC1" t="inlineStr">
+        <is>
+          <t>minutes_trend</t>
+        </is>
+      </c>
+      <c r="DD1" t="inlineStr">
+        <is>
+          <t>role_type_encoded</t>
+        </is>
+      </c>
+      <c r="DE1" t="inlineStr">
+        <is>
+          <t>dominance_pct</t>
+        </is>
+      </c>
+      <c r="DF1" t="inlineStr">
+        <is>
+          <t>specialization_rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>11036007</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>224015</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sarah strong|CONN</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sarah Strong</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>sarah strong</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CONN</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SCAR</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>CONN</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SCAR</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Pts+Rebs</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>pr</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>25.5</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-04-03T19:00:00.000-04:00</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>148432</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>CONN</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Pts+Rebs</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>25.5</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>28.0</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>31.0</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>23.0</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>26.0</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>27.0</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>30.2</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>30.2</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="AX2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="BE2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="BH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="BL2" t="n">
+        <v>27</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="BQ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>27</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>1.411489234785374</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>0.4484641144988664</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>0.5880681872367859</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>0.08806818723678589</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>0.4484641144988664</v>
+      </c>
+      <c r="CF2" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="CG2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="CI2" t="inlineStr">
+        <is>
+          <t>No spread data: 0.97x default</t>
+        </is>
+      </c>
+      <c r="CJ2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="CK2" t="inlineStr">
+        <is>
+          <t>SCAR</t>
+        </is>
+      </c>
+      <c r="CL2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CM2" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="CN2" t="inlineStr">
+        <is>
+          <t>OVER</t>
+        </is>
+      </c>
+      <c r="CO2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="CX2" t="n">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>0.4484641144988664</v>
+      </c>
+      <c r="CZ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA2" t="n">
+        <v>3</v>
+      </c>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD2" t="n">
+        <v>2</v>
+      </c>
+      <c r="DE2" t="n">
+        <v>1.216216216216216</v>
+      </c>
+      <c r="DF2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>